<commit_message>
latest changes screenshot fix, Browserstack integration
</commit_message>
<xml_diff>
--- a/src/test/resources/Run_Manager.xlsx
+++ b/src/test/resources/Run_Manager.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOHAMMAD.RAFI\TestAutomation\projects\kabi\agi_KabiProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247F3D64-59C0-48C4-B123-3149F4897FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB92636F-0140-4DAB-A706-55A0CC29F31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuiteDetails" sheetId="1" r:id="rId1"/>
     <sheet name="UserDetails" sheetId="2" r:id="rId2"/>
-    <sheet name="MyInfoDetails" sheetId="3" r:id="rId3"/>
-    <sheet name="ProductDetails" sheetId="4" r:id="rId4"/>
-    <sheet name="CardDetails" sheetId="5" r:id="rId5"/>
+    <sheet name="MyInfoDetails" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="ProductDetails" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="CardDetails" sheetId="5" state="hidden" r:id="rId5"/>
     <sheet name="APIDetails" sheetId="6" r:id="rId6"/>
     <sheet name="HeaderDetails" sheetId="7" r:id="rId7"/>
     <sheet name="RequestPayloadDetails" sheetId="8" r:id="rId8"/>
@@ -26,8 +26,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SuiteDetails!$A$1:$M$3</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -36,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="213">
   <si>
     <t>P_Key</t>
   </si>
@@ -110,9 +121,6 @@
     <t>TC_WEB_2</t>
   </si>
   <si>
-    <t>apiLoginValid</t>
-  </si>
-  <si>
     <t>UserDetails~APIValidUser</t>
   </si>
   <si>
@@ -120,9 +128,6 @@
   </si>
   <si>
     <t>API</t>
-  </si>
-  <si>
-    <t>apiLoginInvalid</t>
   </si>
   <si>
     <t>TC_API_2</t>
@@ -478,12 +483,348 @@
   <si>
     <t>[Login][Api] Login Invalid – User details</t>
   </si>
+  <si>
+    <t>apiLoginValid</t>
+  </si>
+  <si>
+    <t>apiLoginInvalid</t>
+  </si>
+  <si>
+    <t>CAFM- Clubbed API- Create WorkOrder</t>
+  </si>
+  <si>
+    <t>CAFM- Clubbed API- Update WorkOrder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[CAFM][ClubbedAPI] Create Work Order </t>
+  </si>
+  <si>
+    <t xml:space="preserve">[CAFM][ClubbedAPI] Update Work Order </t>
+  </si>
+  <si>
+    <t>RegressionSuite</t>
+  </si>
+  <si>
+    <t>Scenario: Create a new Work Order with valid details
+    Given a user provides valid work order details
+    When the user sends a request to the Create Work Order API
+    Then the system should respond with status code 200
+    And the response should confirm that the work order is created successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Scenario: Update an existing Work Order with valid details
+    Given a user provides valid updates for an existing work order
+    When the user sends a request to the Update Work Order API
+    Then the system should respond with status code 200
+    And the response should confirm that the work order is updated successfully</t>
+  </si>
+  <si>
+    <t>cafmCreateWorkOrder</t>
+  </si>
+  <si>
+    <t>cafmUpdateWorkOrder</t>
+  </si>
+  <si>
+    <t>CreateWorkOrderCAFM</t>
+  </si>
+  <si>
+    <t>CreateWorkOrderCAFM_Request_Payload</t>
+  </si>
+  <si>
+    <t>CreateWorkOrderCAFM_Success</t>
+  </si>
+  <si>
+    <t>UserDetails~CreateWorkOrderCAFM</t>
+  </si>
+  <si>
+    <t>ItemBarCode</t>
+  </si>
+  <si>
+    <t>WorkCategory</t>
+  </si>
+  <si>
+    <t>Discipline</t>
+  </si>
+  <si>
+    <t>RequestorName</t>
+  </si>
+  <si>
+    <t>RequestorEmail</t>
+  </si>
+  <si>
+    <t>RequestorPhone</t>
+  </si>
+  <si>
+    <t>InstructionGroupCode</t>
+  </si>
+  <si>
+    <t>InstructionNote</t>
+  </si>
+  <si>
+    <t>DetailedDescription</t>
+  </si>
+  <si>
+    <t>ShortDescription</t>
+  </si>
+  <si>
+    <t>ExternalReference</t>
+  </si>
+  <si>
+    <t>PropertyName</t>
+  </si>
+  <si>
+    <t>WorkSubCategory</t>
+  </si>
+  <si>
+    <t>AssignedTechnician</t>
+  </si>
+  <si>
+    <t>ResourceId</t>
+  </si>
+  <si>
+    <t>CurrentStatus</t>
+  </si>
+  <si>
+    <t>CurrentSubStatus</t>
+  </si>
+  <si>
+    <t>PriorityLevel</t>
+  </si>
+  <si>
+    <t>IsRecurring</t>
+  </si>
+  <si>
+    <t>PreviousWorkOrderNumber</t>
+  </si>
+  <si>
+    <t>HVAC</t>
+  </si>
+  <si>
+    <t>AC-FOREMAN</t>
+  </si>
+  <si>
+    <t>MRI Waseem K</t>
+  </si>
+  <si>
+    <t>P1-Emergency</t>
+  </si>
+  <si>
+    <t>Main Panel</t>
+  </si>
+  <si>
+    <t>MRI Test</t>
+  </si>
+  <si>
+    <t>/CreateWorkOrder</t>
+  </si>
+  <si>
+    <t>https://api-dev.al-ghurair.com/facilities/workorder/v1</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com</t>
+  </si>
+  <si>
+    <t>{
+  "$schema": "http://json-schema.org/draft-04/schema#",
+  "type": "object",
+  "required": ["Message","Data","IsDownStreamError","IsPartialSuccess"],
+  "properties": {
+    "Message": { "type": "string" },
+    "Data": {
+      "type": "object",
+      "required": ["WorkOrders"],
+      "properties": {
+        "WorkOrders": {
+          "type": "array",
+          "minItems": 1,
+          "items": {
+            "type": "object",
+            "required": ["WorkOrderId","BDETCallerSourceId","TimeRecordId","TaskStatus","ResponseMessage","IsFailed"],
+            "properties": {
+              "WorkOrderId": { "type": "integer" },
+              "BDETCallerSourceId": { "type": "integer" },
+              "TimeRecordId": { "type": "integer" },
+              "TaskStatus": { "type": "string" },
+              "ResponseMessage": { "type": "string" },
+              "IsFailed": { "type": "boolean" }
+            },
+            "additionalProperties": true
+          }
+        }
+      },
+      "additionalProperties": true
+    },
+    "ErrorDetails": { "type": ["object","string","null"] },
+    "IsDownStreamError": { "type": "boolean" },
+    "IsPartialSuccess": { "type": "boolean" }
+  },
+  "additionalProperties": true
+}</t>
+  </si>
+  <si>
+    <t>TC_API_3</t>
+  </si>
+  <si>
+    <t>TC_API_4</t>
+  </si>
+  <si>
+    <t>CAFM_Headers_With_ApiKey</t>
+  </si>
+  <si>
+    <t>{ "Content-Type": "application/json", "Ocp-Apim-Subscription-Key": "49f2d2571f5a48a38d507e39236fa606"}</t>
+  </si>
+  <si>
+    <t>LoginValid</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>09ca7a8caa2046e48e1363eaa263f3a6</t>
+  </si>
+  <si>
+    <t>WorkScheduledDate</t>
+  </si>
+  <si>
+    <t>CreatedDateUtc</t>
+  </si>
+  <si>
+    <t>Air conditioner is not cooling properly</t>
+  </si>
+  <si>
+    <t>Check compressor and clean filters</t>
+  </si>
+  <si>
+    <t>SRN-223weq</t>
+  </si>
+  <si>
+    <t>abcd@xyz.com</t>
+  </si>
+  <si>
+    <t>AC not cooling</t>
+  </si>
+  <si>
+    <t>Initial assessment</t>
+  </si>
+  <si>
+    <t>2025-08-15T11:28:00Z</t>
+  </si>
+  <si>
+    <t>2025-07-15T11:28:00Z</t>
+  </si>
+  <si>
+    <t>Ocp-Apim-Subscription-Key</t>
+  </si>
+  <si>
+    <t>{
+  "WorkOrders": [
+    {
+      "WorkCategory": "{WorkCategory}",
+      "ItemBarCode": "{ItemBarCode}",
+      "DetailedDescription": "{DetailedDescription}",
+      "InstructionGroupCode": "{InstructionGroupCode}",
+      "InstructionNote": "{InstructionNote}",
+      "ExternalReference": "{ExternalReference}",
+      "Discipline": "{Discipline}",
+      "RequestorName": "{RequestorName}",
+      "RequestorEmail": "{RequestorEmail}",
+      "RequestorPhone": "{RequestorPhone}",
+      "ShortDescription": "{ShortDescription}",
+      "PropertyName": "{PropertyName}",
+      "WorkSubCategory": "{WorkSubCategory}",
+      "AssignedTechnician": "{AssignedTechnician}",
+      "ResourceId": "{ResourceId}",
+      "WorkItemDetail": {
+        "CurrentStatus": "{CurrentStatus}",
+        "CurrentSubStatus": "{CurrentSubStatus}",
+        "PriorityLevel": "{PriorityLevel}",
+        "IsRecurring": {IsRecurring},
+        "PreviousWorkOrderNumber": "{PreviousWorkOrderNumber}",
+        "WorkScheduledDate": "{WorkScheduledDate}",
+        "CreatedDateUtc": "{CreatedDateUtc}"
+      }
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>ExpectedNodePresent</t>
+  </si>
+  <si>
+    <t>Data.WorkOrders[0].ResponseMessage,
+Data.WorkOrders[0].IsFailed</t>
+  </si>
+  <si>
+    <t>ExpectedFieldsJSON</t>
+  </si>
+  <si>
+    <t>{"Data.WorkOrders[0].ResponseMessage":"contains:Work Order created successfully"})</t>
+  </si>
+  <si>
+    <t>ExtractJSON</t>
+  </si>
+  <si>
+    <t>{ "WorkOrderId": "Data.WorkOrders[0].WorkOrderId" }</t>
+  </si>
+  <si>
+    <t>CAFM-CreateWorkOrder-E2E</t>
+  </si>
+  <si>
+    <t>[CAFM][E2E][API][WebUI] Work Order Create &amp; Verify</t>
+  </si>
+  <si>
+    <t>Scenario: Create a new Work Order via API and verify on CAFM web portal
+    Given a user provides valid work order details
+    When the user sends a request to the Create Work Order API
+    Then the system should respond with status code 200
+    And the response should confirm that the work order is created successfully
+    When the user logs into the CAFM web portal
+    And searches for the created Work Order using the WorkOrderId
+    Then the Work Order should be displayed on the portal
+    And the details on the portal should match the API request and response values</t>
+  </si>
+  <si>
+    <t>cafmWOCreateVerifyWebUI</t>
+  </si>
+  <si>
+    <t>UserDetails~CafmWebPortalLogin</t>
+  </si>
+  <si>
+    <t>CafmWebPortalLogin</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>https://uatcafm.agfacilities.com/Evolution/!System/Security/Login.aspx?ReturnUrl=%2fEvolution%2f!System%2fTasks%2fF_TASKS%2fViewF_TASKSItems.aspx%3f</t>
+  </si>
+  <si>
+    <t>EVOLUTION_WS_API</t>
+  </si>
+  <si>
+    <t>Welcome@123</t>
+  </si>
+  <si>
+    <t>TC_Web_3</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>cafmtestcheck</t>
+  </si>
+  <si>
+    <t>https://opensource-demo.orangehrmlive.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -544,8 +885,30 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -576,8 +939,14 @@
         <bgColor rgb="FF339966"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FF339966"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -613,31 +982,17 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -686,12 +1041,77 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Hyperlink 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -703,13 +1123,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1125,388 +1538,546 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" style="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="47" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" style="21" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.5703125" style="7"/>
+    <col min="1" max="1" width="10" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="45.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.5703125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="M1" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="17.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="18" t="s">
+      <c r="B2" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="18"/>
-      <c r="J2" s="19" t="s">
+      <c r="I2" s="16"/>
+      <c r="J2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19" t="s">
+      <c r="K2" s="17"/>
+      <c r="L2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="75">
-      <c r="A3" s="6">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K3" s="7">
+        <v>1</v>
+      </c>
+      <c r="L3" s="7">
+        <v>1</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="60">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K4" s="7">
+        <v>1</v>
+      </c>
+      <c r="L4" s="7">
+        <v>2</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" s="27" customFormat="1" ht="75">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D5" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K5" s="28">
+        <v>1</v>
+      </c>
+      <c r="L5" s="28">
+        <v>3</v>
+      </c>
+      <c r="M5" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" s="27" customFormat="1" ht="75">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="7" t="s">
+      <c r="E6" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K6" s="28">
+        <v>1</v>
+      </c>
+      <c r="L6" s="28">
+        <v>4</v>
+      </c>
+      <c r="M6" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="75">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="7">
+        <v>1</v>
+      </c>
+      <c r="L7" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="75">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="7">
+        <v>1</v>
+      </c>
+      <c r="L8" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="75">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="7">
+        <v>1</v>
+      </c>
+      <c r="L9" s="7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="135">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J10" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1</v>
+      </c>
+      <c r="L10" s="7">
+        <v>8</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="150">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J11" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K11" s="7">
+        <v>1</v>
+      </c>
+      <c r="L11" s="7">
+        <v>9</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="240">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J3" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="9">
+      <c r="I12" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J12" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K12" s="7">
         <v>1</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L12" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J13" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="K13" s="7">
         <v>1</v>
       </c>
-      <c r="M3" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="60">
-      <c r="A4" s="6">
-        <v>2</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J4" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="9">
-        <v>1</v>
-      </c>
-      <c r="L4" s="9">
-        <v>2</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="75">
-      <c r="A5" s="6">
-        <v>3</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J5" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="9">
-        <v>1</v>
-      </c>
-      <c r="L5" s="9">
-        <v>3</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="60">
-      <c r="A6" s="6">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J6" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="9">
-        <v>1</v>
-      </c>
-      <c r="L6" s="9">
-        <v>4</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="75">
-      <c r="A7" s="6">
-        <v>5</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J7" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="K7" s="9">
-        <v>1</v>
-      </c>
-      <c r="L7" s="9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="75">
-      <c r="A8" s="6">
-        <v>6</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J8" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="K8" s="9">
-        <v>1</v>
-      </c>
-      <c r="L8" s="9">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="75">
-      <c r="A9" s="6">
-        <v>7</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="J9" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="K9" s="9">
-        <v>1</v>
-      </c>
-      <c r="L9" s="9">
-        <v>7</v>
+      <c r="L13" s="7">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="E1:E2 F1">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1516,117 +2087,315 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:AD10"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="16" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="26.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="19.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="29.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:30">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>205</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="I1" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="K1" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="L1" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="M1" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="N1" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="O1" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="P1" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q1" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="R1" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="S1" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="T1" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="U1" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="V1" s="29" t="s">
+        <v>157</v>
+      </c>
+      <c r="W1" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="X1" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="Y1" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="Z1" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="AA1" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="AB1" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="AC1" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="AD1" s="29" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30">
+      <c r="A2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" s="41" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30">
+      <c r="A3" t="s">
         <v>116</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F3" s="5">
+      <c r="B3" s="41" t="s">
+        <v>212</v>
+      </c>
+      <c r="F3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G3" s="3">
         <v>11111111</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:30">
       <c r="A4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="F4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="E4" t="s">
+    </row>
+    <row r="5" spans="1:30">
+      <c r="A5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="F5" t="s">
         <v>109</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C5" s="10"/>
-      <c r="E5" t="s">
-        <v>111</v>
-      </c>
-      <c r="F5" s="5">
+      <c r="G5" s="3">
         <v>11111111</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:30">
       <c r="A6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3114791</v>
+      </c>
+      <c r="D6" s="3">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30">
+      <c r="A7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1234567</v>
+      </c>
+      <c r="D7" s="3">
+        <v>123456</v>
+      </c>
+      <c r="E7" s="3">
+        <v>111111</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:30">
+      <c r="A8" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="5">
+      <c r="C8" s="3">
         <v>3114791</v>
       </c>
-      <c r="C6" s="5">
-        <v>123456</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3">
+        <v>111111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" s="21" customFormat="1" ht="30">
+      <c r="A9" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="H9" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="I9" s="35">
+        <v>1234567890</v>
+      </c>
+      <c r="J9" s="35" t="s">
+        <v>183</v>
+      </c>
+      <c r="K9" s="35">
+        <v>31</v>
+      </c>
+      <c r="L9" s="35" t="s">
+        <v>184</v>
+      </c>
+      <c r="M9" s="35" t="s">
+        <v>185</v>
+      </c>
+      <c r="N9" s="35" t="s">
+        <v>164</v>
+      </c>
+      <c r="O9" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="P9" s="35" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q9" s="35">
         <v>1234567</v>
       </c>
-      <c r="C7" s="5">
-        <v>123456</v>
-      </c>
-      <c r="D7" s="5">
-        <v>111111</v>
-      </c>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" s="5">
-        <v>3114791</v>
-      </c>
-      <c r="C8" s="5"/>
+      <c r="R9" s="35" t="s">
+        <v>187</v>
+      </c>
+      <c r="S9" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="T9" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="U9" s="35" t="s">
+        <v>168</v>
+      </c>
+      <c r="V9" s="35">
+        <v>6</v>
+      </c>
+      <c r="W9" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="X9" s="35"/>
+      <c r="Y9" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="Z9" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="AA9" s="35"/>
+      <c r="AB9" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="AC9" s="35" t="s">
+        <v>190</v>
+      </c>
+      <c r="AD9" s="22" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" ht="45">
+      <c r="A10" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="39" t="s">
+        <v>207</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>208</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{0F66BBAE-6821-479C-95D7-F39B391C6F43}"/>
+    <hyperlink ref="G10" r:id="rId2" xr:uid="{090CC6EE-7BA4-4ACA-8F92-EE7A7A25461B}"/>
+    <hyperlink ref="B2" r:id="rId3" xr:uid="{4015D0D7-5D1C-4B78-8894-17A669F1A5E7}"/>
+    <hyperlink ref="B3" r:id="rId4" xr:uid="{BC11A2D0-C8B6-4E49-A1BA-75EC78256B9D}"/>
+  </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>
@@ -1643,57 +2412,57 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
         <v>34</v>
-      </c>
-      <c r="C2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
       </c>
       <c r="E2">
         <v>101</v>
@@ -1711,13 +2480,13 @@
         <v>5565665456</v>
       </c>
       <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" t="s">
         <v>47</v>
-      </c>
-      <c r="K2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L2" t="s">
-        <v>49</v>
       </c>
       <c r="M2" t="s">
         <v>19</v>
@@ -1745,21 +2514,21 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1767,10 +2536,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -1778,10 +2547,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1789,10 +2558,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -1816,21 +2585,21 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C2">
         <v>234</v>
@@ -1848,82 +2617,128 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" style="22" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="22" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" style="22" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" style="22" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="22" customWidth="1"/>
+    <col min="6" max="6" width="25.5703125" style="22" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" style="22" customWidth="1"/>
+    <col min="8" max="16384" width="11.5703125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:7" ht="30">
+      <c r="A1" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="30">
+      <c r="A2" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
+      <c r="C2" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="E2" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="30">
+      <c r="A3" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B3" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="22" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3" t="s">
-        <v>74</v>
-      </c>
+    <row r="4" spans="1:7" ht="30">
+      <c r="A4" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="31"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="31"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{8D5B4A40-888E-4D99-949C-FD04A5FE0E00}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{67153EBC-DE8A-4333-AFD5-7D0749755E57}"/>
+    <hyperlink ref="D3" r:id="rId3" xr:uid="{0D92B396-13F9-490F-A7EC-A88F1DA96FA7}"/>
+  </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>
@@ -1935,27 +2750,35 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" customWidth="1"/>
-    <col min="2" max="2" width="29.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" style="22" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" style="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>75</v>
+      <c r="A1" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="60">
-      <c r="A2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>76</v>
+      <c r="A2" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="75">
+      <c r="A3" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1970,27 +2793,35 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="39.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="83.7109375" style="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="90">
-      <c r="A2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>78</v>
+      <c r="A1" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="60">
+      <c r="A2" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="409.5">
+      <c r="A3" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2005,61 +2836,104 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="28.85546875" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" customWidth="1"/>
+    <col min="1" max="1" width="22.85546875" style="22" customWidth="1"/>
+    <col min="2" max="5" width="37.5703125" style="34" customWidth="1"/>
+    <col min="6" max="6" width="46.5703125" style="22" customWidth="1"/>
+    <col min="7" max="7" width="48" style="22" customWidth="1"/>
+    <col min="8" max="8" width="59.140625" style="22" customWidth="1"/>
+    <col min="9" max="16384" width="11.5703125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="G1" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="180">
+      <c r="A2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="25"/>
+      <c r="H2" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="255">
-      <c r="A2" t="s">
+    <row r="3" spans="1:8" ht="180">
+      <c r="A3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="3" t="s">
+      <c r="B3" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="25"/>
+      <c r="H3" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="255">
-      <c r="A3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" t="s">
-        <v>87</v>
+    </row>
+    <row r="4" spans="1:8" ht="409.5">
+      <c r="A4" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>196</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>198</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="B5" s="34" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes to the logger and api methods
</commit_message>
<xml_diff>
--- a/src/test/resources/Run_Manager.xlsx
+++ b/src/test/resources/Run_Manager.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOHAMMAD.RAFI\TestAutomation\projects\kabi\agi_KabiProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB92636F-0140-4DAB-A706-55A0CC29F31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D556AD9-9A6A-4691-8284-8CEDC7C261ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuiteDetails" sheetId="1" r:id="rId1"/>
     <sheet name="UserDetails" sheetId="2" r:id="rId2"/>
-    <sheet name="MyInfoDetails" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="ProductDetails" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="CardDetails" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="APIDetails" sheetId="6" r:id="rId6"/>
-    <sheet name="HeaderDetails" sheetId="7" r:id="rId7"/>
-    <sheet name="RequestPayloadDetails" sheetId="8" r:id="rId8"/>
-    <sheet name="ResponseDetails" sheetId="9" r:id="rId9"/>
+    <sheet name="RelyAppApis" sheetId="10" r:id="rId3"/>
+    <sheet name="MyInfoDetails" sheetId="3" state="hidden" r:id="rId4"/>
+    <sheet name="ProductDetails" sheetId="4" state="hidden" r:id="rId5"/>
+    <sheet name="CardDetails" sheetId="5" state="hidden" r:id="rId6"/>
+    <sheet name="APIDetails" sheetId="6" r:id="rId7"/>
+    <sheet name="HeaderDetails" sheetId="7" r:id="rId8"/>
+    <sheet name="RequestPayloadDetails" sheetId="8" r:id="rId9"/>
+    <sheet name="ResponseDetails" sheetId="9" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SuiteDetails!$A$1:$M$3</definedName>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="247">
   <si>
     <t>P_Key</t>
   </si>
@@ -680,9 +681,6 @@
     <t>false</t>
   </si>
   <si>
-    <t>.</t>
-  </si>
-  <si>
     <t>09ca7a8caa2046e48e1363eaa263f3a6</t>
   </si>
   <si>
@@ -754,14 +752,7 @@
     <t>ExpectedNodePresent</t>
   </si>
   <si>
-    <t>Data.WorkOrders[0].ResponseMessage,
-Data.WorkOrders[0].IsFailed</t>
-  </si>
-  <si>
     <t>ExpectedFieldsJSON</t>
-  </si>
-  <si>
-    <t>{"Data.WorkOrders[0].ResponseMessage":"contains:Work Order created successfully"})</t>
   </si>
   <si>
     <t>ExtractJSON</t>
@@ -811,20 +802,160 @@
     <t>TC_Web_3</t>
   </si>
   <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>cafmtestcheck</t>
-  </si>
-  <si>
     <t>https://opensource-demo.orangehrmlive.com</t>
+  </si>
+  <si>
+    <t>addEmergencyContact</t>
+  </si>
+  <si>
+    <t>TC_API_5</t>
+  </si>
+  <si>
+    <t>[AGFS][API] Add Emergency Contact</t>
+  </si>
+  <si>
+    <t>2616e11f450a4109851c8148b5b4bd35</t>
+  </si>
+  <si>
+    <t>BirthDate</t>
+  </si>
+  <si>
+    <t>2000-03-01T12:00:00Z</t>
+  </si>
+  <si>
+    <t>BirthCountry</t>
+  </si>
+  <si>
+    <t>Pakistan</t>
+  </si>
+  <si>
+    <t>AE</t>
+  </si>
+  <si>
+    <t>test1</t>
+  </si>
+  <si>
+    <t>test2</t>
+  </si>
+  <si>
+    <t>Sister</t>
+  </si>
+  <si>
+    <t>Work Mobile Phone</t>
+  </si>
+  <si>
+    <t>IsEmergencyContact</t>
+  </si>
+  <si>
+    <t>CountryCode</t>
+  </si>
+  <si>
+    <t>PhoneNumber</t>
+  </si>
+  <si>
+    <t>PrimaryFlag</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>AddEmergencyContact</t>
+  </si>
+  <si>
+    <t>AddEmergencyContact_Success</t>
+  </si>
+  <si>
+    <t>AddEmergencyContact_Request_Payload</t>
+  </si>
+  <si>
+    <t>/{employeeNumber}/contacts/create</t>
+  </si>
+  <si>
+    <t>https://api-uat.al-ghurair.com/humanresource/employee/v1</t>
+  </si>
+  <si>
+    <t>Add Emergency Contact for AGFS Employee Rely App by employee number</t>
+  </si>
+  <si>
+    <t>RelyAppApis~AddEmergencyContact</t>
+  </si>
+  <si>
+    <t>RelyApp_Headers_With_ApiKey</t>
+  </si>
+  <si>
+    <t>{ "Content-Type": "application/json", "Ocp-Apim-Subscription-Key": "2616e11f450a4109851c8148b5b4bd35"}</t>
+  </si>
+  <si>
+    <t>Data.RelationshipInfo[0].Type,Data.RelationshipInfo[0].IsEmergencyContact</t>
+  </si>
+  <si>
+    <t>{"Message":"contains:Emergency Contact added successfully"})</t>
+  </si>
+  <si>
+    <t>{ "Id": "Data.RelationshipInfo[0].Id" }</t>
+  </si>
+  <si>
+    <t>Rely-APIs-AddEmergencyContact</t>
+  </si>
+  <si>
+    <t>Message,Data.WorkOrders[0].ResponseMessage,
+Data.WorkOrders[0].IsFailed</t>
+  </si>
+  <si>
+    <t>{
+  "Message": "Work Order operation completed",
+  "Data.WorkOrders[0].ResponseMessage": "contains:Work Order created successfully"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">employeeNumber </t>
+  </si>
+  <si>
+    <t>Relationship_Type</t>
+  </si>
+  <si>
+    <t>Names_LegislationCode</t>
+  </si>
+  <si>
+    <t>Phone_Type</t>
+  </si>
+  <si>
+    <t>Relationship_LegislationCode</t>
+  </si>
+  <si>
+    <t>{
+  "BirthDate": "{BirthDate}",
+  "BirthCountry": "{BirthCountry}",
+  "names": [
+    {
+      "LegislationCode": "{Names_LegislationCode}",
+      "LastName": "{LastName}",
+      "FirstName": "{FirstName}"
+    }
+  ],
+  "contactRelationships": [
+    {
+      "Type": "{Relationship_Type}",
+      "LegislationCode": "{Relationship_LegislationCode}",
+      "IsEmergencyContact": {IsEmergencyContact}
+    }
+  ],
+  "phones": [
+    {
+      "Type": "{Phone_Type}",
+      "CountryCode": "{CountryCode}",
+      "PhoneNumber": "{PhoneNumber}",
+      "PrimaryFlag": {PrimaryFlag}
+    }
+  ]
+}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -907,6 +1038,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -988,7 +1125,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1104,7 +1241,30 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -1824,7 +1984,7 @@
         <v>105</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>19</v>
+        <v>115</v>
       </c>
       <c r="K7" s="7">
         <v>1</v>
@@ -1862,7 +2022,7 @@
         <v>105</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>19</v>
+        <v>115</v>
       </c>
       <c r="K8" s="7">
         <v>1</v>
@@ -1900,7 +2060,7 @@
         <v>105</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>19</v>
+        <v>115</v>
       </c>
       <c r="K9" s="7">
         <v>1</v>
@@ -1996,22 +2156,22 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>203</v>
-      </c>
       <c r="G12" s="5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>18</v>
@@ -2026,45 +2186,45 @@
         <v>1</v>
       </c>
       <c r="L12" s="7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="15.75">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="30">
       <c r="A13" s="4">
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>210</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>209</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>134</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K13" s="7">
         <v>1</v>
       </c>
       <c r="L13" s="7">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -2085,13 +2245,142 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.85546875" style="22" customWidth="1"/>
+    <col min="2" max="5" width="37.5703125" style="34" customWidth="1"/>
+    <col min="6" max="6" width="46.5703125" style="22" customWidth="1"/>
+    <col min="7" max="7" width="48" style="22" customWidth="1"/>
+    <col min="8" max="8" width="59.140625" style="22" customWidth="1"/>
+    <col min="9" max="16384" width="11.5703125" style="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="G1" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="38" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="180">
+      <c r="A2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="25"/>
+      <c r="H2" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="180">
+      <c r="A3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="25"/>
+      <c r="H3" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="409.5">
+      <c r="A4" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>240</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="409.5">
+      <c r="A5" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AD10"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.5703125" customWidth="1"/>
+    <col min="2" max="2" width="58.5703125" style="43" customWidth="1"/>
     <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -2124,8 +2413,8 @@
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>205</v>
+      <c r="B1" s="41" t="s">
+        <v>202</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>87</v>
@@ -2203,21 +2492,21 @@
         <v>162</v>
       </c>
       <c r="AB1" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="AC1" s="29" t="s">
         <v>181</v>
       </c>
-      <c r="AC1" s="29" t="s">
-        <v>182</v>
-      </c>
       <c r="AD1" s="29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:30">
       <c r="A2" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="41" t="s">
-        <v>212</v>
+      <c r="B2" s="42" t="s">
+        <v>207</v>
       </c>
       <c r="F2" t="s">
         <v>109</v>
@@ -2230,8 +2519,8 @@
       <c r="A3" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="41" t="s">
-        <v>212</v>
+      <c r="B3" s="42" t="s">
+        <v>207</v>
       </c>
       <c r="F3" t="s">
         <v>109</v>
@@ -2306,6 +2595,7 @@
       <c r="A9" s="21" t="s">
         <v>139</v>
       </c>
+      <c r="B9" s="22"/>
       <c r="H9" s="35" t="s">
         <v>163</v>
       </c>
@@ -2313,16 +2603,16 @@
         <v>1234567890</v>
       </c>
       <c r="J9" s="35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K9" s="35">
         <v>31</v>
       </c>
       <c r="L9" s="35" t="s">
+        <v>183</v>
+      </c>
+      <c r="M9" s="35" t="s">
         <v>184</v>
-      </c>
-      <c r="M9" s="35" t="s">
-        <v>185</v>
       </c>
       <c r="N9" s="35" t="s">
         <v>164</v>
@@ -2331,13 +2621,13 @@
         <v>165</v>
       </c>
       <c r="P9" s="35" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q9" s="35">
         <v>1234567</v>
       </c>
       <c r="R9" s="35" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="S9" s="35" t="s">
         <v>166</v>
@@ -2352,7 +2642,7 @@
         <v>6</v>
       </c>
       <c r="W9" s="35" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="X9" s="35"/>
       <c r="Y9" s="35" t="s">
@@ -2363,30 +2653,30 @@
       </c>
       <c r="AA9" s="35"/>
       <c r="AB9" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="AC9" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="AC9" s="35" t="s">
-        <v>190</v>
-      </c>
       <c r="AD9" s="22" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:30" ht="45">
       <c r="A10" s="21" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
       <c r="F10" s="39" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2406,90 +2696,125 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="11.7109375" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65C58635-1506-4A14-A92D-991A8F7E2B6C}">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25" style="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="34" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.42578125" style="34" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5703125" style="34" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="29" style="34" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="11.5703125" style="34"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:16" ht="45">
+      <c r="A1" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>241</v>
+      </c>
+      <c r="D1" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>243</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2">
-        <v>101</v>
-      </c>
-      <c r="F2">
-        <v>123456</v>
-      </c>
-      <c r="G2">
-        <v>231568645</v>
-      </c>
-      <c r="H2">
-        <v>78879</v>
-      </c>
-      <c r="I2">
-        <v>5565665456</v>
-      </c>
-      <c r="J2" t="s">
-        <v>45</v>
-      </c>
-      <c r="K2" t="s">
-        <v>46</v>
-      </c>
-      <c r="L2" t="s">
-        <v>47</v>
-      </c>
-      <c r="M2" t="s">
-        <v>19</v>
+      <c r="I1" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="J1" s="48" t="s">
+        <v>245</v>
+      </c>
+      <c r="K1" s="32" t="s">
+        <v>221</v>
+      </c>
+      <c r="L1" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="M1" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="N1" s="32" t="s">
+        <v>223</v>
+      </c>
+      <c r="O1" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="P1" s="44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="30">
+      <c r="A2" s="34" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="34">
+        <v>90029806</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="47" t="s">
+        <v>216</v>
+      </c>
+      <c r="G2" s="34" t="s">
+        <v>217</v>
+      </c>
+      <c r="H2" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="I2" s="47" t="s">
+        <v>219</v>
+      </c>
+      <c r="J2" s="47" t="s">
+        <v>216</v>
+      </c>
+      <c r="K2" s="47" t="s">
+        <v>225</v>
+      </c>
+      <c r="L2" s="34" t="s">
+        <v>220</v>
+      </c>
+      <c r="M2" s="34">
+        <v>971</v>
+      </c>
+      <c r="N2" s="34">
+        <v>8687123456</v>
+      </c>
+      <c r="O2" s="47" t="s">
+        <v>225</v>
+      </c>
+      <c r="P2" s="46" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2503,6 +2828,103 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultColWidth="11.7109375" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2">
+        <v>101</v>
+      </c>
+      <c r="F2">
+        <v>123456</v>
+      </c>
+      <c r="G2">
+        <v>231568645</v>
+      </c>
+      <c r="H2">
+        <v>78879</v>
+      </c>
+      <c r="I2">
+        <v>5565665456</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
@@ -2573,7 +2995,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
@@ -2615,16 +3037,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.140625" style="22" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" style="22" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" style="22" customWidth="1"/>
-    <col min="4" max="4" width="33.85546875" style="22" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="22" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" style="22" customWidth="1"/>
+    <col min="4" max="4" width="39.7109375" style="22" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" style="22" customWidth="1"/>
     <col min="6" max="6" width="25.5703125" style="22" customWidth="1"/>
     <col min="7" max="7" width="20.5703125" style="22" customWidth="1"/>
     <col min="8" max="16384" width="11.5703125" style="22"/>
@@ -2722,10 +3144,28 @@
         <v>141</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
+    <row r="5" spans="1:7" ht="45">
+      <c r="A5" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>230</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>229</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="31"/>
@@ -2738,6 +3178,7 @@
     <hyperlink ref="D4" r:id="rId1" xr:uid="{8D5B4A40-888E-4D99-949C-FD04A5FE0E00}"/>
     <hyperlink ref="D2" r:id="rId2" xr:uid="{67153EBC-DE8A-4333-AFD5-7D0749755E57}"/>
     <hyperlink ref="D3" r:id="rId3" xr:uid="{0D92B396-13F9-490F-A7EC-A88F1DA96FA7}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{4479E6E8-E15C-4B50-8451-3DFD0C93776D}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2748,9 +3189,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.85546875" style="22" customWidth="1"/>
@@ -2781,47 +3222,12 @@
         <v>176</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="39.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="83.7109375" style="21" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="60">
-      <c r="A2" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="409.5">
-      <c r="A3" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>192</v>
+    <row r="4" spans="1:2" ht="75">
+      <c r="A4" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -2835,105 +3241,44 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" style="22" customWidth="1"/>
-    <col min="2" max="5" width="37.5703125" style="34" customWidth="1"/>
-    <col min="6" max="6" width="46.5703125" style="22" customWidth="1"/>
-    <col min="7" max="7" width="48" style="22" customWidth="1"/>
-    <col min="8" max="8" width="59.140625" style="22" customWidth="1"/>
-    <col min="9" max="16384" width="11.5703125" style="22"/>
+    <col min="1" max="1" width="39.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="83.7109375" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1" s="32" t="s">
-        <v>193</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>195</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="G1" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="H1" s="38" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="180">
-      <c r="A2" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B2" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="25"/>
-      <c r="H2" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="180">
-      <c r="A3" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="G3" s="25"/>
-      <c r="H3" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="409.5">
-      <c r="A4" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>81</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>194</v>
-      </c>
-      <c r="D4" s="36" t="s">
-        <v>196</v>
-      </c>
-      <c r="E4" s="36" t="s">
-        <v>198</v>
-      </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="B5" s="34" t="s">
-        <v>179</v>
+      <c r="B1" s="20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="60">
+      <c r="A2" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="409.5">
+      <c r="A3" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="390">
+      <c r="A4" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new changes on api agfs rely api scenarios
</commit_message>
<xml_diff>
--- a/src/test/resources/Run_Manager.xlsx
+++ b/src/test/resources/Run_Manager.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOHAMMAD.RAFI\TestAutomation\projects\kabi\agi_KabiProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D556AD9-9A6A-4691-8284-8CEDC7C261ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221F6678-428C-49E9-842F-791F225E4864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="SuiteDetails" sheetId="1" r:id="rId1"/>
-    <sheet name="UserDetails" sheetId="2" r:id="rId2"/>
+    <sheet name="SuiteDetails3" sheetId="11" r:id="rId1"/>
+    <sheet name="SuiteDetails" sheetId="1" r:id="rId2"/>
     <sheet name="RelyAppApis" sheetId="10" r:id="rId3"/>
     <sheet name="MyInfoDetails" sheetId="3" state="hidden" r:id="rId4"/>
     <sheet name="ProductDetails" sheetId="4" state="hidden" r:id="rId5"/>
@@ -23,9 +23,13 @@
     <sheet name="HeaderDetails" sheetId="7" r:id="rId8"/>
     <sheet name="RequestPayloadDetails" sheetId="8" r:id="rId9"/>
     <sheet name="ResponseDetails" sheetId="9" r:id="rId10"/>
+    <sheet name="UserDetails" sheetId="2" r:id="rId11"/>
+    <sheet name="SuiteDetails (2)" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SuiteDetails!$A$1:$M$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SuiteDetails!$A$1:$M$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'SuiteDetails (2)'!$A$1:$M$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SuiteDetails3!$A$1:$M$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="359">
   <si>
     <t>P_Key</t>
   </si>
@@ -366,15 +370,6 @@
   </si>
   <si>
     <t>UserDetails~InvalidOtp</t>
-  </si>
-  <si>
-    <t>[Login][Mobile] Verify successful login with valid Driver ID</t>
-  </si>
-  <si>
-    <t>[Login][Mobile] Verify error on login with invalid Driver ID</t>
-  </si>
-  <si>
-    <t>[Login][Mobile] Verify OTP error for invalid or expired input</t>
   </si>
   <si>
     <t>Scenario: Login with valid Driver ID on Mobile
@@ -808,9 +803,6 @@
     <t>addEmergencyContact</t>
   </si>
   <si>
-    <t>TC_API_5</t>
-  </si>
-  <si>
     <t>[AGFS][API] Add Emergency Contact</t>
   </si>
   <si>
@@ -874,9 +866,6 @@
     <t>https://api-uat.al-ghurair.com/humanresource/employee/v1</t>
   </si>
   <si>
-    <t>Add Emergency Contact for AGFS Employee Rely App by employee number</t>
-  </si>
-  <si>
     <t>RelyAppApis~AddEmergencyContact</t>
   </si>
   <si>
@@ -889,13 +878,7 @@
     <t>Data.RelationshipInfo[0].Type,Data.RelationshipInfo[0].IsEmergencyContact</t>
   </si>
   <si>
-    <t>{"Message":"contains:Emergency Contact added successfully"})</t>
-  </si>
-  <si>
     <t>{ "Id": "Data.RelationshipInfo[0].Id" }</t>
-  </si>
-  <si>
-    <t>Rely-APIs-AddEmergencyContact</t>
   </si>
   <si>
     <t>Message,Data.WorkOrders[0].ResponseMessage,
@@ -950,12 +933,504 @@
   ]
 }</t>
   </si>
+  <si>
+    <t>100000003889128</t>
+  </si>
+  <si>
+    <t>{"Message":"contains:Emergency Contact Added successfully"})</t>
+  </si>
+  <si>
+    <t>/{employeeNumber}</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeDetails</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeDetails_Request_Payload</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeDetails_Success</t>
+  </si>
+  <si>
+    <t>[AGFS][API] Retrieve Employee Details</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Details for AGFS Employee Rely App by employee number</t>
+  </si>
+  <si>
+    <t>Add Emergency Contact for AGFS Employee Rely App by related employeenumber of employee number</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeDetails</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeDetails</t>
+  </si>
+  <si>
+    <t>phones</t>
+  </si>
+  <si>
+    <t>names</t>
+  </si>
+  <si>
+    <t>addresses</t>
+  </si>
+  <si>
+    <t>emails</t>
+  </si>
+  <si>
+    <t>workRelationships.assignments</t>
+  </si>
+  <si>
+    <t>{"Message":"contains:Employee Detail Retrieved successfully"})</t>
+  </si>
+  <si>
+    <t>Data.EmployeeId,Data.EmployeeNumber</t>
+  </si>
+  <si>
+    <t>{ "Id": "Data.EmployeeId" }</t>
+  </si>
+  <si>
+    <t>{
+  "Details": [
+    "{Detail1}",
+    "{Detail2}",
+    "{Detail3}",
+    "{Detail4}",
+    "{Detail5}"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>Detail1</t>
+  </si>
+  <si>
+    <t>Detail2</t>
+  </si>
+  <si>
+    <t>Detail3</t>
+  </si>
+  <si>
+    <t>Detail4</t>
+  </si>
+  <si>
+    <t>Detail5</t>
+  </si>
+  <si>
+    <t>[AGFS][API] Retrieve Emergency Contacts Detail</t>
+  </si>
+  <si>
+    <t>Retrieve Emergency Contacts Detail for AGFS Employee Rely App by employee number</t>
+  </si>
+  <si>
+    <t>retrieveEmergencyContactsDetail</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmergencyContactsDetail</t>
+  </si>
+  <si>
+    <t>RetrieveEmergencyContactsDetail</t>
+  </si>
+  <si>
+    <t>contactRelationships</t>
+  </si>
+  <si>
+    <t>Detail6</t>
+  </si>
+  <si>
+    <t>Detail7</t>
+  </si>
+  <si>
+    <t>Detail8</t>
+  </si>
+  <si>
+    <t>RetrieveEmergencyContactsDetail_Request_Payload</t>
+  </si>
+  <si>
+    <t>RetrieveEmergencyContactsDetail_Success</t>
+  </si>
+  <si>
+    <t>/{employeeNumber}/contacts</t>
+  </si>
+  <si>
+    <t>{
+  "Details": [
+    "{Detail6}",
+    "{Detail7}",
+    "{Detail8}"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>Message,Data.EmergencyContacts.RelationshipInfo[0].Id</t>
+  </si>
+  <si>
+    <t>{"Message":"contains:Emergency Contacts Retrieved successfully"})</t>
+  </si>
+  <si>
+    <t>{ "Id": "Data.EmergencyContacts.RelationshipInfo[0].Id" }</t>
+  </si>
+  <si>
+    <t>Rely-APIs-HumanResource.Employee</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecord_Request_Payload</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecord_Success</t>
+  </si>
+  <si>
+    <t>recordType</t>
+  </si>
+  <si>
+    <t>attachments</t>
+  </si>
+  <si>
+    <t>Passport</t>
+  </si>
+  <si>
+    <t>Details_RetrieveEmployeeRecord</t>
+  </si>
+  <si>
+    <t>{
+  "Details": [
+    "{Details_RetrieveEmployeeRecord}"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{"Message":"contains:Record details retrieved successfully"})</t>
+  </si>
+  <si>
+    <t>{ "Id": "Data.Records.RecordNumber" }</t>
+  </si>
+  <si>
+    <t>/{employeeNumber}/documents/{recordType}</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Passport for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Emirates ID for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Passport</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Emirates ID</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordPassPort</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordEmiratesID</t>
+  </si>
+  <si>
+    <t>TC_API_5</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordPassport</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordEmiratesId</t>
+  </si>
+  <si>
+    <t>Emirates ID</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordEmiratesId</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordPassport</t>
+  </si>
+  <si>
+    <t>Residence Visa</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordResidenceVisa</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Residence Visa</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Residence Visa for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordResidenceVisa</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordResidenceVisa</t>
+  </si>
+  <si>
+    <t>TC_API_6</t>
+  </si>
+  <si>
+    <t>documentRecordsDFF</t>
+  </si>
+  <si>
+    <t>Details_documentRecordsDFF</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordResidenceVisa_Request_Payload</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordResidenceVisa_Success</t>
+  </si>
+  <si>
+    <t>Message,Data.RecordType,Data.Records.RecordNumber</t>
+  </si>
+  <si>
+    <t>{
+  "Details":[
+ "{Details_RetrieveEmployeeRecord}","{Details_documentRecordsDFF}"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Salary Certificate</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Salary Certificate for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordSalaryCertificate</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordSalaryCertificate</t>
+  </si>
+  <si>
+    <t>TC_API_7</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordSalaryCertificate</t>
+  </si>
+  <si>
+    <t>Salary Certificate</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordSalaryCertificate_Success</t>
+  </si>
+  <si>
+    <t>Message,Data.RecordType,Data.Records.Attachments.AttachmentId</t>
+  </si>
+  <si>
+    <t>{ "Id": "Data.Records.Attachments.AttachmentId" }</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Drivers License for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Drivers License</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordDriversLicense</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordDriversLicense</t>
+  </si>
+  <si>
+    <t>TC_API_8</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordDriversLicense</t>
+  </si>
+  <si>
+    <t>Drivers License</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordDriversLicense_Success</t>
+  </si>
+  <si>
+    <t>Health Insurance</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Health Insurance</t>
+  </si>
+  <si>
+    <t>[AGFS][API] 
+Retrieve Employee Record - For Work Permit</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Work Permit for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>Retrieve Employee Record for Health Insurance for AGFS Employee Rely App</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordHealthInsurance</t>
+  </si>
+  <si>
+    <t>retrieveEmployeeRecordWorkPermit</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordHealthInsurance</t>
+  </si>
+  <si>
+    <t>RelyAppApis~RetrieveEmployeeRecordWorkPermit</t>
+  </si>
+  <si>
+    <t>TC_API_9</t>
+  </si>
+  <si>
+    <t>TC_API_10</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordHealthInsurance</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordWorkPermit</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordWorkPermit_Success</t>
+  </si>
+  <si>
+    <t>RetrieveEmployeeRecordHealthInsurance_Success</t>
+  </si>
+  <si>
+    <t>Message,Data.RecordType,Data.Records.RecordId</t>
+  </si>
+  <si>
+    <t>Work Permit</t>
+  </si>
+  <si>
+    <t>{ "RecordType":"Data.RecordType","Id": "Data.Records.RecordId" }</t>
+  </si>
+  <si>
+    <t>Rely-APIs-HumanResource.Employee - Emergency Contact</t>
+  </si>
+  <si>
+    <t>Rely-APIs-HumanResource.Employee - Information</t>
+  </si>
+  <si>
+    <t>Rely-APIs-HumanResource.Employee - Documents</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[Login][Mobile] Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>successful login</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>valid Driver ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[Login][Mobile] Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>error on login</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>invalid Driver ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[Login][Mobile] Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>OTP error</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>invalid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> or expired input</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1044,8 +1519,27 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Open Sans"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1080,6 +1574,66 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor rgb="FF339966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor rgb="FF339966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor rgb="FF339966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor rgb="FF339966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1125,7 +1679,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1262,8 +1816,69 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1271,7 +1886,63 @@
     <cellStyle name="Hyperlink 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF9C0006"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF9C0006"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1697,7 +2368,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4474903F-2FD0-41D4-9E87-8659D3498B46}">
   <dimension ref="A1:M13"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
@@ -1705,8 +2376,8 @@
     <col min="2" max="2" width="26.28515625" style="6" customWidth="1"/>
     <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
     <col min="4" max="4" width="45.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="47" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="51.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" style="5" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" style="5" bestFit="1" customWidth="1"/>
@@ -1791,200 +2462,188 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="75">
+    <row r="3" spans="1:13" ht="45">
       <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>15</v>
+        <v>353</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>124</v>
+        <v>206</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>120</v>
+        <v>248</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>16</v>
+        <v>205</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>111</v>
+        <v>227</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="J3" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K3" s="7">
         <v>1</v>
       </c>
       <c r="L3" s="7">
-        <v>1</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="45">
       <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>15</v>
+        <v>354</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>125</v>
+        <v>246</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>123</v>
+        <v>247</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>21</v>
+        <v>249</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>117</v>
+        <v>250</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K4" s="7">
         <v>1</v>
       </c>
       <c r="L4" s="7">
-        <v>2</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" s="27" customFormat="1" ht="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="45">
       <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="F5" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="27" t="s">
+      <c r="B5" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="27" t="s">
-        <v>105</v>
+      <c r="I5" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="K5" s="28">
+        <v>19</v>
+      </c>
+      <c r="K5" s="7">
         <v>1</v>
       </c>
-      <c r="L5" s="28">
+      <c r="L5" s="7">
         <v>3</v>
       </c>
-      <c r="M5" s="27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" s="27" customFormat="1" ht="75">
+    </row>
+    <row r="6" spans="1:13" ht="45">
       <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="27" t="s">
+      <c r="B6" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="H6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="27" t="s">
-        <v>105</v>
+      <c r="I6" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="K6" s="28">
+        <v>19</v>
+      </c>
+      <c r="K6" s="7">
         <v>1</v>
       </c>
-      <c r="L6" s="28">
+      <c r="L6" s="7">
         <v>4</v>
       </c>
-      <c r="M6" s="27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="75">
+    </row>
+    <row r="7" spans="1:13" ht="45">
       <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>15</v>
+        <v>355</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>97</v>
+        <v>295</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>100</v>
+        <v>293</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>88</v>
+        <v>297</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>91</v>
+        <v>302</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>28</v>
+        <v>298</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K7" s="7">
         <v>1</v>
@@ -1993,36 +2652,36 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="75">
+    <row r="8" spans="1:13" ht="45">
       <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>15</v>
+        <v>355</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>98</v>
+        <v>306</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>101</v>
+        <v>307</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>89</v>
+        <v>308</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>22</v>
+        <v>309</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>30</v>
+        <v>310</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K8" s="7">
         <v>1</v>
@@ -2031,36 +2690,36 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="75">
+    <row r="9" spans="1:13" ht="45">
       <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>104</v>
+        <v>355</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>99</v>
+        <v>317</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>102</v>
+        <v>318</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>93</v>
+        <v>319</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>96</v>
+        <v>320</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>103</v>
+        <v>321</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K9" s="7">
         <v>1</v>
@@ -2069,36 +2728,36 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="135">
+    <row r="10" spans="1:13" ht="45">
       <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>130</v>
+        <v>355</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>132</v>
+        <v>328</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>135</v>
+        <v>327</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>137</v>
+        <v>329</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>142</v>
+        <v>330</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>173</v>
+        <v>331</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>26</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J10" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K10" s="7">
         <v>1</v>
@@ -2106,40 +2765,37 @@
       <c r="L10" s="7">
         <v>8</v>
       </c>
-      <c r="M10" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="150">
+    </row>
+    <row r="11" spans="1:13" ht="45">
       <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>131</v>
+        <v>355</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>133</v>
+        <v>336</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>136</v>
+        <v>339</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>138</v>
+        <v>340</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>118</v>
+        <v>342</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>174</v>
+        <v>344</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>26</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K11" s="7">
         <v>1</v>
@@ -2147,40 +2803,37 @@
       <c r="L11" s="7">
         <v>9</v>
       </c>
-      <c r="M11" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="240">
+    </row>
+    <row r="12" spans="1:13" ht="45">
       <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>196</v>
+        <v>355</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>197</v>
+        <v>337</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>198</v>
+        <v>338</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>199</v>
+        <v>341</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>200</v>
+        <v>343</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>206</v>
+        <v>345</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="K12" s="7">
         <v>1</v>
@@ -2189,54 +2842,19 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="30">
-      <c r="A13" s="4">
-        <v>11</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="J13" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="7">
-        <v>1</v>
-      </c>
-      <c r="L13" s="7">
-        <v>11</v>
-      </c>
+    <row r="13" spans="1:13" ht="16.5">
+      <c r="A13" s="63"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="E1:E2 F1">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2247,11 +2865,13 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.85546875" style="22" customWidth="1"/>
-    <col min="2" max="5" width="37.5703125" style="34" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="37.5703125" style="34" customWidth="1"/>
     <col min="6" max="6" width="46.5703125" style="22" customWidth="1"/>
     <col min="7" max="7" width="48" style="22" customWidth="1"/>
     <col min="8" max="8" width="59.140625" style="22" customWidth="1"/>
@@ -2266,13 +2886,13 @@
         <v>77</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F1" s="24" t="s">
         <v>80</v>
@@ -2284,11 +2904,11 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="180">
+    <row r="2" spans="1:8" ht="180" hidden="1">
       <c r="A2" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="48" t="s">
         <v>81</v>
       </c>
       <c r="C2" s="33"/>
@@ -2302,11 +2922,11 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="180">
+    <row r="3" spans="1:8" ht="180" hidden="1">
       <c r="A3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="48" t="s">
         <v>81</v>
       </c>
       <c r="C3" s="33"/>
@@ -2322,47 +2942,205 @@
     </row>
     <row r="4" spans="1:8" ht="409.5">
       <c r="A4" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="49" t="s">
         <v>81</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="25"/>
       <c r="H4" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="409.5">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30">
       <c r="A5" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="B5" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="B5" s="49" t="s">
         <v>81</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="25"/>
-      <c r="H5" s="6" t="s">
-        <v>172</v>
-      </c>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" ht="30">
+      <c r="A6" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>256</v>
+      </c>
+      <c r="E6" s="36" t="s">
+        <v>258</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" ht="45">
+      <c r="A7" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>278</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>279</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>280</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" ht="30">
+      <c r="A8" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" ht="45">
+      <c r="A9" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" ht="45">
+      <c r="A10" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B10" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>325</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>326</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:8" ht="45">
+      <c r="A11" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>325</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E11" s="36" t="s">
+        <v>326</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" ht="45">
+      <c r="A12" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>350</v>
+      </c>
+      <c r="D12" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E12" s="36" t="s">
+        <v>352</v>
+      </c>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" ht="30">
+      <c r="A13" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>350</v>
+      </c>
+      <c r="D13" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E13" s="36" t="s">
+        <v>352</v>
+      </c>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -2374,7 +3152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AD10"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
@@ -2414,7 +3192,7 @@
         <v>31</v>
       </c>
       <c r="B1" s="41" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>87</v>
@@ -2426,104 +3204,104 @@
         <v>95</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="H1" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="I1" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="K1" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="L1" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="M1" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="N1" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="O1" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="P1" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="I1" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="J1" s="29" t="s">
+      <c r="Q1" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="R1" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="S1" s="29" t="s">
         <v>151</v>
       </c>
-      <c r="K1" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="L1" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="M1" s="29" t="s">
+      <c r="T1" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="U1" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="N1" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="O1" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="P1" s="29" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q1" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="R1" s="29" t="s">
-        <v>152</v>
-      </c>
-      <c r="S1" s="29" t="s">
+      <c r="V1" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="T1" s="29" t="s">
+      <c r="W1" s="29" t="s">
         <v>155</v>
       </c>
-      <c r="U1" s="29" t="s">
+      <c r="X1" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="V1" s="29" t="s">
+      <c r="Y1" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="W1" s="29" t="s">
+      <c r="Z1" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="X1" s="29" t="s">
+      <c r="AA1" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="Y1" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="Z1" s="29" t="s">
-        <v>161</v>
-      </c>
-      <c r="AA1" s="29" t="s">
-        <v>162</v>
-      </c>
       <c r="AB1" s="29" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AC1" s="29" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AD1" s="29" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:30">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:30">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G3" s="3">
         <v>11111111</v>
@@ -2531,23 +3309,23 @@
     </row>
     <row r="4" spans="1:30">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D4" s="8"/>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:30">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D5" s="8"/>
       <c r="F5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G5" s="3">
         <v>11111111</v>
@@ -2593,90 +3371,90 @@
     </row>
     <row r="9" spans="1:30" s="21" customFormat="1" ht="30">
       <c r="A9" s="21" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B9" s="22"/>
       <c r="H9" s="35" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I9" s="35">
         <v>1234567890</v>
       </c>
       <c r="J9" s="35" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K9" s="35">
         <v>31</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="M9" s="35" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="N9" s="35" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="O9" s="35" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="P9" s="35" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="Q9" s="35">
         <v>1234567</v>
       </c>
       <c r="R9" s="35" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="S9" s="35" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="T9" s="35" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="U9" s="35" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="V9" s="35">
         <v>6</v>
       </c>
       <c r="W9" s="35" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="X9" s="35"/>
       <c r="Y9" s="35" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="Z9" s="37" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="AA9" s="35"/>
       <c r="AB9" s="35" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="AC9" s="35" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AD9" s="22" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:30" ht="45">
       <c r="A10" s="21" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
       <c r="F10" s="39" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2695,129 +3473,1658 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5680339F-F732-4ED6-9EE4-86BAB403DD41}">
+  <dimension ref="A1:M15"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="45.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.5703125" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="17.25">
+      <c r="A2" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="75">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="7">
+        <v>1</v>
+      </c>
+      <c r="L3" s="7">
+        <v>1</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="60">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="7">
+        <v>1</v>
+      </c>
+      <c r="L4" s="7">
+        <v>2</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" s="27" customFormat="1" ht="75">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K5" s="28">
+        <v>1</v>
+      </c>
+      <c r="L5" s="28">
+        <v>3</v>
+      </c>
+      <c r="M5" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" s="27" customFormat="1" ht="75">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K6" s="28">
+        <v>1</v>
+      </c>
+      <c r="L6" s="28">
+        <v>4</v>
+      </c>
+      <c r="M6" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="75">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="7">
+        <v>1</v>
+      </c>
+      <c r="L7" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="75">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="7">
+        <v>1</v>
+      </c>
+      <c r="L8" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="75">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="7">
+        <v>1</v>
+      </c>
+      <c r="L9" s="7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="135">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J10" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1</v>
+      </c>
+      <c r="L10" s="7">
+        <v>8</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="150">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J11" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K11" s="7">
+        <v>1</v>
+      </c>
+      <c r="L11" s="7">
+        <v>9</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="240">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J12" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K12" s="7">
+        <v>1</v>
+      </c>
+      <c r="L12" s="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="45">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J13" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K13" s="7">
+        <v>1</v>
+      </c>
+      <c r="L13" s="7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="30">
+      <c r="A14" s="4">
+        <v>12</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J14" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K14" s="7">
+        <v>1</v>
+      </c>
+      <c r="L14" s="7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="30">
+      <c r="A15" s="4">
+        <v>13</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J15" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K15" s="7">
+        <v>1</v>
+      </c>
+      <c r="L15" s="7">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="E1:E2 F1">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="45.85546875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="45.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.5703125" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="17.25">
+      <c r="A2" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="75">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="66" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="66" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K3" s="7">
+        <v>1</v>
+      </c>
+      <c r="L3" s="7">
+        <v>1</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="60">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="66" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="66" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="68" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K4" s="7">
+        <v>1</v>
+      </c>
+      <c r="L4" s="7">
+        <v>2</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="75">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="65" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="65" t="s">
+        <v>356</v>
+      </c>
+      <c r="D5" s="69" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" s="7">
+        <v>1</v>
+      </c>
+      <c r="L5" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="75">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="65" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="65" t="s">
+        <v>357</v>
+      </c>
+      <c r="D6" s="69" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" s="7">
+        <v>1</v>
+      </c>
+      <c r="L6" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="75">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="65" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="65" t="s">
+        <v>358</v>
+      </c>
+      <c r="D7" s="69" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="7">
+        <v>1</v>
+      </c>
+      <c r="L7" s="7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="45">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="64" t="s">
+        <v>353</v>
+      </c>
+      <c r="C8" s="67" t="s">
+        <v>206</v>
+      </c>
+      <c r="D8" s="64" t="s">
+        <v>248</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K8" s="7">
+        <v>1</v>
+      </c>
+      <c r="L8" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="45">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="64" t="s">
+        <v>354</v>
+      </c>
+      <c r="C9" s="67" t="s">
+        <v>246</v>
+      </c>
+      <c r="D9" s="64" t="s">
+        <v>247</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K9" s="7">
+        <v>1</v>
+      </c>
+      <c r="L9" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="45">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="64" t="s">
+        <v>353</v>
+      </c>
+      <c r="C10" s="67" t="s">
+        <v>265</v>
+      </c>
+      <c r="D10" s="64" t="s">
+        <v>266</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J10" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1</v>
+      </c>
+      <c r="L10" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="45">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C11" s="67" t="s">
+        <v>294</v>
+      </c>
+      <c r="D11" s="64" t="s">
+        <v>292</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J11" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K11" s="7">
+        <v>1</v>
+      </c>
+      <c r="L11" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="45">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="B12" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C12" s="67" t="s">
+        <v>295</v>
+      </c>
+      <c r="D12" s="64" t="s">
+        <v>293</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J12" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K12" s="7">
+        <v>1</v>
+      </c>
+      <c r="L12" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="45">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+      <c r="B13" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C13" s="67" t="s">
+        <v>306</v>
+      </c>
+      <c r="D13" s="64" t="s">
+        <v>307</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J13" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K13" s="7">
+        <v>1</v>
+      </c>
+      <c r="L13" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="45">
+      <c r="A14" s="4">
+        <v>12</v>
+      </c>
+      <c r="B14" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C14" s="67" t="s">
+        <v>317</v>
+      </c>
+      <c r="D14" s="64" t="s">
+        <v>318</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J14" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K14" s="7">
+        <v>1</v>
+      </c>
+      <c r="L14" s="7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="45">
+      <c r="A15" s="4">
+        <v>13</v>
+      </c>
+      <c r="B15" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C15" s="67" t="s">
+        <v>328</v>
+      </c>
+      <c r="D15" s="64" t="s">
+        <v>327</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J15" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K15" s="7">
+        <v>1</v>
+      </c>
+      <c r="L15" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="45">
+      <c r="A16" s="4">
+        <v>14</v>
+      </c>
+      <c r="B16" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C16" s="67" t="s">
+        <v>336</v>
+      </c>
+      <c r="D16" s="64" t="s">
+        <v>339</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J16" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K16" s="7">
+        <v>1</v>
+      </c>
+      <c r="L16" s="7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="45">
+      <c r="A17" s="4">
+        <v>15</v>
+      </c>
+      <c r="B17" s="64" t="s">
+        <v>355</v>
+      </c>
+      <c r="C17" s="67" t="s">
+        <v>337</v>
+      </c>
+      <c r="D17" s="64" t="s">
+        <v>338</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J17" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="K17" s="7">
+        <v>1</v>
+      </c>
+      <c r="L17" s="7">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="E1:E2 F1">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65C58635-1506-4A14-A92D-991A8F7E2B6C}">
-  <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <dimension ref="A1:AA11"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="25" style="34" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.42578125" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" style="34" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" style="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="34" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" style="34" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.42578125" style="34" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" style="34" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" style="34" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5703125" style="34" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="34" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29" style="34" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="11.5703125" style="34"/>
+    <col min="1" max="1" width="39.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" style="34" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="34" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" style="34" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" style="34" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="17" max="20" width="11.5703125" style="34"/>
+    <col min="21" max="21" width="19.42578125" style="34" customWidth="1"/>
+    <col min="22" max="22" width="19.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="11.5703125" style="34"/>
+    <col min="25" max="25" width="16.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="31.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="28" style="34" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="11.5703125" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="45">
+    <row r="1" spans="1:27" ht="15.75" customHeight="1">
       <c r="A1" s="32" t="s">
         <v>31</v>
       </c>
       <c r="B1" s="44" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C1" s="44" t="s">
-        <v>241</v>
+        <v>187</v>
       </c>
       <c r="D1" s="44" t="s">
+        <v>234</v>
+      </c>
+      <c r="E1" s="56" t="s">
+        <v>208</v>
+      </c>
+      <c r="F1" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="G1" s="57" t="s">
+        <v>236</v>
+      </c>
+      <c r="H1" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="57" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="57" t="s">
+        <v>235</v>
+      </c>
+      <c r="K1" s="58" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="M1" s="57" t="s">
+        <v>237</v>
+      </c>
+      <c r="N1" s="57" t="s">
+        <v>218</v>
+      </c>
+      <c r="O1" s="57" t="s">
+        <v>219</v>
+      </c>
+      <c r="P1" s="57" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q1" s="51" t="s">
+        <v>260</v>
+      </c>
+      <c r="R1" s="51" t="s">
+        <v>261</v>
+      </c>
+      <c r="S1" s="51" t="s">
+        <v>262</v>
+      </c>
+      <c r="T1" s="51" t="s">
+        <v>263</v>
+      </c>
+      <c r="U1" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="V1" s="54" t="s">
+        <v>271</v>
+      </c>
+      <c r="W1" s="54" t="s">
+        <v>272</v>
+      </c>
+      <c r="X1" s="54" t="s">
+        <v>273</v>
+      </c>
+      <c r="Y1" s="59" t="s">
+        <v>284</v>
+      </c>
+      <c r="Z1" s="59" t="s">
+        <v>287</v>
+      </c>
+      <c r="AA1" s="61" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A2" s="55" t="s">
+        <v>222</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>240</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>209</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>211</v>
+      </c>
+      <c r="G2" s="47" t="s">
         <v>212</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="H2" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="I2" s="34" t="s">
         <v>214</v>
       </c>
-      <c r="F1" s="32" t="s">
+      <c r="J2" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="K2" s="47" t="s">
+        <v>212</v>
+      </c>
+      <c r="L2" s="47" t="s">
+        <v>221</v>
+      </c>
+      <c r="M2" s="34" t="s">
+        <v>216</v>
+      </c>
+      <c r="N2" s="34">
+        <v>971</v>
+      </c>
+      <c r="O2" s="34">
+        <v>8687123456</v>
+      </c>
+      <c r="P2" s="47" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A3" s="52" t="s">
         <v>243</v>
       </c>
-      <c r="G1" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="32" t="s">
-        <v>242</v>
-      </c>
-      <c r="J1" s="48" t="s">
-        <v>245</v>
-      </c>
-      <c r="K1" s="32" t="s">
-        <v>221</v>
-      </c>
-      <c r="L1" s="32" t="s">
-        <v>244</v>
-      </c>
-      <c r="M1" s="32" t="s">
-        <v>222</v>
-      </c>
-      <c r="N1" s="32" t="s">
-        <v>223</v>
-      </c>
-      <c r="O1" s="32" t="s">
-        <v>224</v>
-      </c>
-      <c r="P1" s="44" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="30">
-      <c r="A2" s="34" t="s">
-        <v>226</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="34">
+      <c r="B3" s="45"/>
+      <c r="C3" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" s="47">
         <v>90029806</v>
       </c>
-      <c r="D2" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>215</v>
-      </c>
-      <c r="F2" s="47" t="s">
-        <v>216</v>
-      </c>
-      <c r="G2" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="H2" s="34" t="s">
-        <v>218</v>
-      </c>
-      <c r="I2" s="47" t="s">
-        <v>219</v>
-      </c>
-      <c r="J2" s="47" t="s">
-        <v>216</v>
-      </c>
-      <c r="K2" s="47" t="s">
-        <v>225</v>
-      </c>
-      <c r="L2" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="M2" s="34">
-        <v>971</v>
-      </c>
-      <c r="N2" s="34">
-        <v>8687123456</v>
-      </c>
-      <c r="O2" s="47" t="s">
-        <v>225</v>
-      </c>
-      <c r="P2" s="46" t="s">
-        <v>211</v>
+      <c r="G3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="34" t="s">
+        <v>251</v>
+      </c>
+      <c r="R3" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="S3" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="T3" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="U3" s="34" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A4" s="53" t="s">
+        <v>269</v>
+      </c>
+      <c r="C4" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D4" s="47">
+        <v>90029806</v>
+      </c>
+      <c r="V4" s="34" t="s">
+        <v>270</v>
+      </c>
+      <c r="W4" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="X4" s="34" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A5" s="50" t="s">
+        <v>299</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D5" s="47">
+        <v>90029806</v>
+      </c>
+      <c r="Y5" s="34" t="s">
+        <v>286</v>
+      </c>
+      <c r="Z5" s="34" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A6" s="50" t="s">
+        <v>300</v>
+      </c>
+      <c r="C6" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D6" s="60">
+        <v>90037461</v>
+      </c>
+      <c r="Y6" s="34" t="s">
+        <v>301</v>
+      </c>
+      <c r="Z6" s="34" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A7" s="61" t="s">
+        <v>305</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D7" s="60">
+        <v>90037461</v>
+      </c>
+      <c r="Y7" s="34" t="s">
+        <v>304</v>
+      </c>
+      <c r="Z7" s="34" t="s">
+        <v>285</v>
+      </c>
+      <c r="AA7" s="34" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A8" s="50" t="s">
+        <v>322</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D8" s="60">
+        <v>90007690</v>
+      </c>
+      <c r="Y8" s="34" t="s">
+        <v>323</v>
+      </c>
+      <c r="Z8" s="34" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A9" s="50" t="s">
+        <v>332</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="34">
+        <v>90035700</v>
+      </c>
+      <c r="Y9" s="34" t="s">
+        <v>333</v>
+      </c>
+      <c r="Z9" s="34" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A10" s="50" t="s">
+        <v>346</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D10" s="34">
+        <v>90035700</v>
+      </c>
+      <c r="Y10" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="Z10" s="34" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" ht="15.75" customHeight="1">
+      <c r="A11" s="50" t="s">
+        <v>347</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D11" s="34">
+        <v>90029806</v>
+      </c>
+      <c r="Y11" s="34" t="s">
+        <v>351</v>
+      </c>
+      <c r="Z11" s="34" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>
@@ -3039,20 +5346,20 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.140625" style="22" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" style="22" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" style="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" style="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.42578125" style="22" customWidth="1"/>
-    <col min="4" max="4" width="39.7109375" style="22" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" style="22" customWidth="1"/>
-    <col min="6" max="6" width="25.5703125" style="22" customWidth="1"/>
-    <col min="7" max="7" width="20.5703125" style="22" customWidth="1"/>
+    <col min="4" max="4" width="56.140625" style="22" customWidth="1"/>
+    <col min="5" max="5" width="43.7109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="47.140625" style="22" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="11.5703125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1">
       <c r="A1" s="23" t="s">
         <v>31</v>
       </c>
@@ -3075,9 +5382,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30">
+    <row r="2" spans="1:7" ht="15.75" hidden="1" customHeight="1">
       <c r="A2" s="22" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>66</v>
@@ -3086,7 +5393,7 @@
         <v>67</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>68</v>
@@ -3098,7 +5405,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30">
+    <row r="3" spans="1:7" ht="15.75" hidden="1" customHeight="1">
       <c r="A3" s="22" t="s">
         <v>71</v>
       </c>
@@ -3109,7 +5416,7 @@
         <v>67</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>68</v>
@@ -3121,57 +5428,258 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30">
+    <row r="4" spans="1:7" ht="15.75" hidden="1" customHeight="1">
       <c r="A4" s="22" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>66</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" customHeight="1">
       <c r="A5" s="22" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>66</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="F5" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A6" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="G5" s="22" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="31"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="31"/>
+      <c r="D6" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>244</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A7" s="31" t="s">
+        <v>269</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>276</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>274</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A8" s="22" t="s">
+        <v>299</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A9" s="22" t="s">
+        <v>300</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A10" s="22" t="s">
+        <v>305</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F10" s="62" t="s">
+        <v>313</v>
+      </c>
+      <c r="G10" s="62" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A11" s="22" t="s">
+        <v>322</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A12" s="22" t="s">
+        <v>332</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A13" s="22" t="s">
+        <v>346</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A14" s="22" t="s">
+        <v>347</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>348</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3179,6 +5687,15 @@
     <hyperlink ref="D2" r:id="rId2" xr:uid="{67153EBC-DE8A-4333-AFD5-7D0749755E57}"/>
     <hyperlink ref="D3" r:id="rId3" xr:uid="{0D92B396-13F9-490F-A7EC-A88F1DA96FA7}"/>
     <hyperlink ref="D5" r:id="rId4" xr:uid="{4479E6E8-E15C-4B50-8451-3DFD0C93776D}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{FE4E3984-C281-40F4-940D-8DD20CB78E85}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{0859CA03-DD2C-4657-BBA3-2BC270D84DC3}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{466AFE03-7388-4E62-9A9E-47A291FE0A4E}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{0C89AD67-512B-4E03-B896-28480DD19551}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{883B1328-5AFC-4A18-B31A-873217FEFD04}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{2C00480B-6488-4C68-8561-FCA671E71F87}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{261A1012-A060-459F-B264-B060E06B2E1B}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{E8BA514F-D7C1-4A44-834E-059A5C9E615D}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{B3D47458-C5BB-412E-B332-0E6B7434E95F}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3216,18 +5733,18 @@
     </row>
     <row r="3" spans="1:2" ht="75">
       <c r="A3" s="22" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="75">
       <c r="A4" s="22" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3242,11 +5759,11 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="83.7109375" style="21" customWidth="1"/>
+    <col min="1" max="1" width="48.7109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.28515625" style="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3267,18 +5784,50 @@
     </row>
     <row r="3" spans="1:2" ht="409.5">
       <c r="A3" s="21" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="390">
       <c r="A4" s="21" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>246</v>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="135">
+      <c r="A5" s="22" t="s">
+        <v>244</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="105">
+      <c r="A6" s="22" t="s">
+        <v>274</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="75">
+      <c r="A7" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="105">
+      <c r="A8" s="22" t="s">
+        <v>313</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>